<commit_message>
Release v0.4.0: hyperparameter tuning and algorithm v2.
Add Validation grid tuning (12_tune_hyperparams), adopt random_forest_v2 and
catboost_v2, algo_id registry and two-step train UI, run_config pipeline
fixes, inference primary/aux alignment, version menu, and tuning docs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/outputs/reports/catboost_v1/evaluation.xlsx
+++ b/outputs/reports/catboost_v1/evaluation.xlsx
@@ -487,37 +487,37 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9880541750552592</v>
+        <v>0.9891878040571551</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2199440820130475</v>
+        <v>0.2240652235029519</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9535353535353536</v>
+        <v>0.9224537037037037</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3574403634986748</v>
+        <v>0.3605519113322778</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9881748762035277</v>
+        <v>0.9894090560245588</v>
       </c>
       <c r="G2" t="n">
-        <v>139889</v>
+        <v>257840</v>
       </c>
       <c r="H2" t="n">
-        <v>1674</v>
+        <v>2760</v>
       </c>
       <c r="I2" t="n">
-        <v>23</v>
+        <v>67</v>
       </c>
       <c r="J2" t="n">
-        <v>472</v>
+        <v>797</v>
       </c>
       <c r="K2" t="n">
-        <v>0.9892893031100048</v>
+        <v>0.9845251209814957</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7598629647128564</v>
+        <v>0.7592751825078895</v>
       </c>
     </row>
   </sheetData>
@@ -613,43 +613,43 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.003484492249644511</v>
+        <v>0.003304470213872656</v>
       </c>
       <c r="C2" t="n">
-        <v>1421</v>
+        <v>2615</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3201970443349754</v>
+        <v>0.297131931166348</v>
       </c>
       <c r="E2" t="n">
-        <v>91.89202368512714</v>
+        <v>89.91817505842363</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9191919191919192</v>
+        <v>0.8993055555555556</v>
       </c>
       <c r="G2" t="n">
-        <v>7103</v>
+        <v>13074</v>
       </c>
       <c r="H2" t="n">
-        <v>0.06799943685766577</v>
+        <v>0.06348477895058896</v>
       </c>
       <c r="I2" t="n">
-        <v>19.51487676995209</v>
+        <v>19.21178731890832</v>
       </c>
       <c r="J2" t="n">
-        <v>0.9757575757575757</v>
+        <v>0.9606481481481481</v>
       </c>
       <c r="K2" t="n">
-        <v>14206</v>
+        <v>26147</v>
       </c>
       <c r="L2" t="n">
-        <v>0.03407011122061101</v>
+        <v>0.03204956591578384</v>
       </c>
       <c r="M2" t="n">
-        <v>9.777640120762745</v>
+        <v>9.698851507644104</v>
       </c>
       <c r="N2" t="n">
-        <v>0.9777777777777777</v>
+        <v>0.9699074074074074</v>
       </c>
     </row>
   </sheetData>
@@ -700,13 +700,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>109618</v>
+        <v>214020</v>
       </c>
       <c r="C2" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="D2" t="n">
-        <v>8.210330420186466e-05</v>
+        <v>9.344921035417251e-05</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -719,13 +719,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>18805</v>
+        <v>30192</v>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0001063546929008242</v>
+        <v>0.0004305776364599894</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -738,13 +738,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7126</v>
+        <v>8851</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D4" t="n">
-        <v>0.000140331181588549</v>
+        <v>0.0014687605920235</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -757,13 +757,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3087</v>
+        <v>3321</v>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="D5" t="n">
-        <v>0.001295756397797214</v>
+        <v>0.004215597711532671</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -776,13 +776,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1272</v>
+        <v>1518</v>
       </c>
       <c r="C6" t="n">
         <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>0.00550314465408805</v>
+        <v>0.00461133069828722</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -795,13 +795,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>571</v>
+        <v>783</v>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D7" t="n">
-        <v>0.008756567425569177</v>
+        <v>0.01915708812260536</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -814,13 +814,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>335</v>
+        <v>505</v>
       </c>
       <c r="C8" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="D8" t="n">
-        <v>0.06865671641791045</v>
+        <v>0.02574257425742574</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -833,13 +833,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>248</v>
+        <v>422</v>
       </c>
       <c r="C9" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D9" t="n">
-        <v>0.07661290322580645</v>
+        <v>0.03317535545023697</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -852,13 +852,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>258</v>
+        <v>473</v>
       </c>
       <c r="C10" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="D10" t="n">
-        <v>0.09689922480620156</v>
+        <v>0.07610993657505286</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -871,13 +871,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>738</v>
+        <v>1379</v>
       </c>
       <c r="C11" t="n">
-        <v>400</v>
+        <v>719</v>
       </c>
       <c r="D11" t="n">
-        <v>0.5420054200542005</v>
+        <v>0.5213923132704859</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Release v0.6.0: GBM/Stacked/EasyEnsemble v2 tuning and registration.
Validation tune for three families, v2 registry and train scripts, and Test adoption on refreshed data. Primary/aux 4x4 comparison deferred to next session.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/outputs/reports/catboost_v1/evaluation.xlsx
+++ b/outputs/reports/catboost_v1/evaluation.xlsx
@@ -487,37 +487,37 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9891878040571551</v>
+        <v>0.9893713857357036</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2240652235029519</v>
+        <v>0.222541690626797</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9224537037037037</v>
+        <v>0.911660777385159</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3605519113322778</v>
+        <v>0.35775363993529</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9894090560245588</v>
+        <v>0.9896245419488517</v>
       </c>
       <c r="G2" t="n">
-        <v>257840</v>
+        <v>257911</v>
       </c>
       <c r="H2" t="n">
-        <v>2760</v>
+        <v>2704</v>
       </c>
       <c r="I2" t="n">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="J2" t="n">
-        <v>797</v>
+        <v>774</v>
       </c>
       <c r="K2" t="n">
-        <v>0.9845251209814957</v>
+        <v>0.9860349941936518</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7592751825078895</v>
+        <v>0.6974527412588878</v>
       </c>
     </row>
   </sheetData>
@@ -613,43 +613,43 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.003304470213872656</v>
+        <v>0.003247100939326255</v>
       </c>
       <c r="C2" t="n">
         <v>2615</v>
       </c>
       <c r="D2" t="n">
-        <v>0.297131931166348</v>
+        <v>0.2860420650095603</v>
       </c>
       <c r="E2" t="n">
-        <v>89.91817505842363</v>
+        <v>88.09152236237887</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8993055555555556</v>
+        <v>0.8810365135453475</v>
       </c>
       <c r="G2" t="n">
         <v>13074</v>
       </c>
       <c r="H2" t="n">
-        <v>0.06348477895058896</v>
+        <v>0.06218448829738412</v>
       </c>
       <c r="I2" t="n">
-        <v>19.21178731890832</v>
+        <v>19.15077155263515</v>
       </c>
       <c r="J2" t="n">
-        <v>0.9606481481481481</v>
+        <v>0.9575971731448764</v>
       </c>
       <c r="K2" t="n">
         <v>26147</v>
       </c>
       <c r="L2" t="n">
-        <v>0.03204956591578384</v>
+        <v>0.03147588633495239</v>
       </c>
       <c r="M2" t="n">
-        <v>9.698851507644104</v>
+        <v>9.693534917175489</v>
       </c>
       <c r="N2" t="n">
-        <v>0.9699074074074074</v>
+        <v>0.9693757361601885</v>
       </c>
     </row>
   </sheetData>
@@ -700,13 +700,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>214020</v>
+        <v>208751</v>
       </c>
       <c r="C2" t="n">
         <v>20</v>
       </c>
       <c r="D2" t="n">
-        <v>9.344921035417251e-05</v>
+        <v>9.580792427341666e-05</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -719,13 +719,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>30192</v>
+        <v>33069</v>
       </c>
       <c r="C3" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0004305776364599894</v>
+        <v>0.000272158214642112</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -738,13 +738,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8851</v>
+        <v>10446</v>
       </c>
       <c r="C4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0014687605920235</v>
+        <v>0.001148765077541643</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -757,13 +757,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3321</v>
+        <v>3979</v>
       </c>
       <c r="C5" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D5" t="n">
-        <v>0.004215597711532671</v>
+        <v>0.004021110831867303</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -776,13 +776,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1518</v>
+        <v>1734</v>
       </c>
       <c r="C6" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="D6" t="n">
-        <v>0.00461133069828722</v>
+        <v>0.01038062283737024</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -795,13 +795,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>783</v>
+        <v>805</v>
       </c>
       <c r="C7" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D7" t="n">
-        <v>0.01915708812260536</v>
+        <v>0.02608695652173913</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -814,13 +814,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>505</v>
+        <v>529</v>
       </c>
       <c r="C8" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D8" t="n">
-        <v>0.02574257425742574</v>
+        <v>0.03402646502835539</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -833,13 +833,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>422</v>
+        <v>446</v>
       </c>
       <c r="C9" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="D9" t="n">
-        <v>0.03317535545023697</v>
+        <v>0.04708520179372197</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -852,13 +852,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>473</v>
+        <v>455</v>
       </c>
       <c r="C10" t="n">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D10" t="n">
-        <v>0.07610993657505286</v>
+        <v>0.1010989010989011</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -871,13 +871,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1379</v>
+        <v>1250</v>
       </c>
       <c r="C11" t="n">
-        <v>719</v>
+        <v>668</v>
       </c>
       <c r="D11" t="n">
-        <v>0.5213923132704859</v>
+        <v>0.5344</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Release v0.7.0: entity-valid tuning, v3 models, and CLI tune pipeline.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/outputs/reports/catboost_v1/evaluation.xlsx
+++ b/outputs/reports/catboost_v1/evaluation.xlsx
@@ -487,37 +487,37 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9893713857357036</v>
+        <v>0.9952022821576764</v>
       </c>
       <c r="C2" t="n">
-        <v>0.222541690626797</v>
+        <v>0.4335260115606936</v>
       </c>
       <c r="D2" t="n">
-        <v>0.911660777385159</v>
+        <v>0.462962962962963</v>
       </c>
       <c r="E2" t="n">
-        <v>0.35775363993529</v>
+        <v>0.4477611940298508</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9896245419488517</v>
+        <v>0.9974477837387364</v>
       </c>
       <c r="G2" t="n">
-        <v>257911</v>
+        <v>38300</v>
       </c>
       <c r="H2" t="n">
-        <v>2704</v>
+        <v>98</v>
       </c>
       <c r="I2" t="n">
+        <v>87</v>
+      </c>
+      <c r="J2" t="n">
         <v>75</v>
       </c>
-      <c r="J2" t="n">
-        <v>774</v>
-      </c>
       <c r="K2" t="n">
-        <v>0.9860349941936518</v>
+        <v>0.8920347896206013</v>
       </c>
       <c r="L2" t="n">
-        <v>0.6974527412588878</v>
+        <v>0.4370031317911339</v>
       </c>
     </row>
   </sheetData>
@@ -613,43 +613,43 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.003247100939326255</v>
+        <v>0.004201244813278008</v>
       </c>
       <c r="C2" t="n">
-        <v>2615</v>
+        <v>386</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2860420650095603</v>
+        <v>0.2461139896373057</v>
       </c>
       <c r="E2" t="n">
-        <v>88.09152236237887</v>
+        <v>58.58120642231177</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8810365135453475</v>
+        <v>0.5864197530864198</v>
       </c>
       <c r="G2" t="n">
-        <v>13074</v>
+        <v>1928</v>
       </c>
       <c r="H2" t="n">
-        <v>0.06218448829738412</v>
+        <v>0.05912863070539419</v>
       </c>
       <c r="I2" t="n">
-        <v>19.15077155263515</v>
+        <v>14.07407407407407</v>
       </c>
       <c r="J2" t="n">
-        <v>0.9575971731448764</v>
+        <v>0.7037037037037037</v>
       </c>
       <c r="K2" t="n">
-        <v>26147</v>
+        <v>3856</v>
       </c>
       <c r="L2" t="n">
-        <v>0.03147588633495239</v>
+        <v>0.03060165975103734</v>
       </c>
       <c r="M2" t="n">
-        <v>9.693534917175489</v>
+        <v>7.283950617283951</v>
       </c>
       <c r="N2" t="n">
-        <v>0.9693757361601885</v>
+        <v>0.7283950617283951</v>
       </c>
     </row>
   </sheetData>
@@ -700,13 +700,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>208751</v>
+        <v>37927</v>
       </c>
       <c r="C2" t="n">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="D2" t="n">
-        <v>9.580792427341666e-05</v>
+        <v>0.001423787802884489</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -719,13 +719,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>33069</v>
+        <v>259</v>
       </c>
       <c r="C3" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D3" t="n">
-        <v>0.000272158214642112</v>
+        <v>0.05405405405405406</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -738,13 +738,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10446</v>
+        <v>99</v>
       </c>
       <c r="C4" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>0.001148765077541643</v>
+        <v>0.0101010101010101</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -757,13 +757,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3979</v>
+        <v>53</v>
       </c>
       <c r="C5" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D5" t="n">
-        <v>0.004021110831867303</v>
+        <v>0.1132075471698113</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -776,13 +776,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1734</v>
+        <v>49</v>
       </c>
       <c r="C6" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D6" t="n">
-        <v>0.01038062283737024</v>
+        <v>0.2448979591836735</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -795,13 +795,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>805</v>
+        <v>20</v>
       </c>
       <c r="C7" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>0.02608695652173913</v>
+        <v>0.15</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -814,13 +814,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>529</v>
+        <v>23</v>
       </c>
       <c r="C8" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D8" t="n">
-        <v>0.03402646502835539</v>
+        <v>0.2173913043478261</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -833,13 +833,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>446</v>
+        <v>18</v>
       </c>
       <c r="C9" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="D9" t="n">
-        <v>0.04708520179372197</v>
+        <v>0.5</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -852,13 +852,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>455</v>
+        <v>33</v>
       </c>
       <c r="C10" t="n">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1010989010989011</v>
+        <v>0.2424242424242424</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -871,13 +871,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1250</v>
+        <v>79</v>
       </c>
       <c r="C11" t="n">
-        <v>668</v>
+        <v>50</v>
       </c>
       <c r="D11" t="n">
-        <v>0.5344</v>
+        <v>0.6329113924050633</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>

</xml_diff>